<commit_message>
Version final con Docker funcionando
</commit_message>
<xml_diff>
--- a/output/resultados.xlsx
+++ b/output/resultados.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,15 +429,10 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Nombres</t>
+          <t>Ubicacion</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
-        <is>
-          <t>Ubicacion</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
         <is>
           <t>Direccion</t>
         </is>
@@ -451,78 +446,25 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Si</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Juan Perez Gomez</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Lima / Lima / Miraflores</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Av. Ejemplo 123</t>
-        </is>
-      </c>
+          <t>Error 500 ONPE</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>87654321</t>
+          <t>74175431</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Maria Torres Ruiz</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Arequipa / Arequipa / Cayma</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Jr. Demo 456</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>45678912</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Si</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Luis Alberto Ramos</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Cusco / Cusco / Wanchaq</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Av. Los Incas 456</t>
-        </is>
-      </c>
+          <t>Error 500 ONPE</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>